<commit_message>
Fichier banque : un seul modèle Banque.xlsx (Journ, Date, Libelle, Debit, Credit, Etat) ; Debit = sortie, Credit = entrée
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8s2z31P3cgDQRDppUofdK
</commit_message>
<xml_diff>
--- a/Imports/modeles/Banque.xlsx
+++ b/Imports/modeles/Banque.xlsx
@@ -437,7 +437,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Jnl</t>
+          <t>Journ</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Solde</t>
+          <t>Etat</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fichier banque : la colonne Etat est supprimée du modèle (Journ, Date, Libelle, Debit, Credit)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8s2z31P3cgDQRDppUofdK
</commit_message>
<xml_diff>
--- a/Imports/modeles/Banque.xlsx
+++ b/Imports/modeles/Banque.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -431,7 +431,6 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,11 +459,6 @@
           <t>Credit</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Etat</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>